<commit_message>
Update and reestructure discussion
</commit_message>
<xml_diff>
--- a/doc/sintesis results literature.xlsx
+++ b/doc/sintesis results literature.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="96">
   <si>
     <t>Author</t>
   </si>
@@ -291,6 +291,30 @@
   </si>
   <si>
     <t>912 plots</t>
+  </si>
+  <si>
+    <t>Hulshob 2013</t>
+  </si>
+  <si>
+    <t>elevation gradient</t>
+  </si>
+  <si>
+    <t>Desert, Tropical, high altitude mediterranean</t>
+  </si>
+  <si>
+    <t>Kraft 2008</t>
+  </si>
+  <si>
+    <t>Amazonia</t>
+  </si>
+  <si>
+    <t>ridges vs valleys</t>
+  </si>
+  <si>
+    <t>1000 sp</t>
+  </si>
+  <si>
+    <t>CWM?</t>
   </si>
 </sst>
 </file>
@@ -608,7 +632,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K46"/>
+  <dimension ref="A1:K52"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.7109375" bestFit="1" customWidth="1"/>
@@ -1499,6 +1523,108 @@
         <v>6</v>
       </c>
     </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>88</v>
+      </c>
+      <c r="B47" t="s">
+        <v>90</v>
+      </c>
+      <c r="C47" t="s">
+        <v>89</v>
+      </c>
+      <c r="E47" t="s">
+        <v>14</v>
+      </c>
+      <c r="F47" t="s">
+        <v>9</v>
+      </c>
+      <c r="G47" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>88</v>
+      </c>
+      <c r="B48" t="s">
+        <v>90</v>
+      </c>
+      <c r="C48" t="s">
+        <v>89</v>
+      </c>
+      <c r="E48" t="s">
+        <v>14</v>
+      </c>
+      <c r="F48" t="s">
+        <v>35</v>
+      </c>
+      <c r="G48" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>88</v>
+      </c>
+      <c r="B49" t="s">
+        <v>90</v>
+      </c>
+      <c r="C49" t="s">
+        <v>89</v>
+      </c>
+      <c r="E49" t="s">
+        <v>30</v>
+      </c>
+      <c r="G49" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>91</v>
+      </c>
+      <c r="B50" t="s">
+        <v>92</v>
+      </c>
+      <c r="C50" t="s">
+        <v>93</v>
+      </c>
+      <c r="D50" t="s">
+        <v>94</v>
+      </c>
+      <c r="E50" t="s">
+        <v>14</v>
+      </c>
+      <c r="F50" t="s">
+        <v>95</v>
+      </c>
+      <c r="H50" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E51" t="s">
+        <v>12</v>
+      </c>
+      <c r="F51" t="s">
+        <v>95</v>
+      </c>
+      <c r="H51" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E52" t="s">
+        <v>3</v>
+      </c>
+      <c r="F52" t="s">
+        <v>95</v>
+      </c>
+      <c r="H52" t="s">
+        <v>5</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J42"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
draft with Lars comments incorporated
</commit_message>
<xml_diff>
--- a/doc/sintesis results literature.xlsx
+++ b/doc/sintesis results literature.xlsx
@@ -15,7 +15,7 @@
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Hoja1!$A$1:$J$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$J$52</definedName>
   </definedNames>
   <calcPr calcId="152511"/>
   <extLst>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="95">
   <si>
     <t>Author</t>
   </si>
@@ -150,9 +150,6 @@
   </si>
   <si>
     <t>No differences between seed bank and vegetation</t>
-  </si>
-  <si>
-    <t>LA</t>
   </si>
   <si>
     <t>convergence</t>
@@ -637,6 +634,7 @@
   <cols>
     <col min="1" max="1" width="22.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="36.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.85546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11.7109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.140625" customWidth="1"/>
     <col min="7" max="8" width="17" bestFit="1" customWidth="1"/>
@@ -645,18 +643,18 @@
     <col min="11" max="11" width="11.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E1" t="s">
         <v>2</v>
@@ -677,18 +675,18 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E2" t="s">
         <v>3</v>
@@ -703,18 +701,18 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E3" t="s">
         <v>3</v>
@@ -729,18 +727,18 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>16</v>
       </c>
       <c r="B4" t="s">
+        <v>68</v>
+      </c>
+      <c r="C4" t="s">
         <v>69</v>
       </c>
-      <c r="C4" t="s">
-        <v>70</v>
-      </c>
       <c r="D4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E4" t="s">
         <v>15</v>
@@ -755,7 +753,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>19</v>
       </c>
@@ -763,10 +761,10 @@
         <v>24</v>
       </c>
       <c r="C5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E5" t="s">
         <v>15</v>
@@ -781,7 +779,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -798,7 +796,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>22</v>
       </c>
@@ -815,7 +813,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>22</v>
       </c>
@@ -832,12 +830,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>22</v>
       </c>
       <c r="B9" t="s">
-        <v>50</v>
+        <v>24</v>
       </c>
       <c r="E9" t="s">
         <v>11</v>
@@ -846,15 +844,18 @@
         <v>35</v>
       </c>
       <c r="G9" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+        <v>46</v>
+      </c>
+      <c r="K9" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>22</v>
       </c>
       <c r="B10" t="s">
-        <v>50</v>
+        <v>24</v>
       </c>
       <c r="E10" t="s">
         <v>14</v>
@@ -863,10 +864,13 @@
         <v>35</v>
       </c>
       <c r="G10" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+        <v>46</v>
+      </c>
+      <c r="K10" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>23</v>
       </c>
@@ -874,7 +878,7 @@
         <v>24</v>
       </c>
       <c r="C11" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E11" t="s">
         <v>14</v>
@@ -886,7 +890,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>23</v>
       </c>
@@ -894,7 +898,7 @@
         <v>24</v>
       </c>
       <c r="C12" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E12" t="s">
         <v>13</v>
@@ -906,7 +910,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>23</v>
       </c>
@@ -914,7 +918,7 @@
         <v>24</v>
       </c>
       <c r="C13" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E13" t="s">
         <v>12</v>
@@ -923,7 +927,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>23</v>
       </c>
@@ -931,7 +935,7 @@
         <v>24</v>
       </c>
       <c r="C14" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E14" t="s">
         <v>30</v>
@@ -940,7 +944,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>23</v>
       </c>
@@ -948,7 +952,7 @@
         <v>24</v>
       </c>
       <c r="C15" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E15" t="s">
         <v>13</v>
@@ -957,10 +961,10 @@
         <v>35</v>
       </c>
       <c r="I15" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>23</v>
       </c>
@@ -968,16 +972,16 @@
         <v>24</v>
       </c>
       <c r="C16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E16" t="s">
-        <v>41</v>
+        <v>12</v>
       </c>
       <c r="F16" t="s">
         <v>35</v>
       </c>
       <c r="I16" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
@@ -988,7 +992,7 @@
         <v>24</v>
       </c>
       <c r="C17" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E17" t="s">
         <v>14</v>
@@ -997,7 +1001,7 @@
         <v>35</v>
       </c>
       <c r="I17" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
@@ -1008,7 +1012,7 @@
         <v>28</v>
       </c>
       <c r="C18" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E18" t="s">
         <v>11</v>
@@ -1028,7 +1032,7 @@
         <v>28</v>
       </c>
       <c r="C19" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E19" t="s">
         <v>13</v>
@@ -1048,7 +1052,7 @@
         <v>28</v>
       </c>
       <c r="C20" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E20" t="s">
         <v>3</v>
@@ -1071,7 +1075,7 @@
         <v>28</v>
       </c>
       <c r="C21" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E21" t="s">
         <v>14</v>
@@ -1091,10 +1095,10 @@
         <v>28</v>
       </c>
       <c r="C22" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E22" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F22" t="s">
         <v>35</v>
@@ -1213,7 +1217,7 @@
         <v>30</v>
       </c>
       <c r="I29" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
@@ -1224,7 +1228,7 @@
         <v>30</v>
       </c>
       <c r="I30" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
@@ -1243,7 +1247,7 @@
         <v>34</v>
       </c>
       <c r="E32" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F32" t="s">
         <v>35</v>
@@ -1257,7 +1261,7 @@
         <v>37</v>
       </c>
       <c r="E33" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F33" t="s">
         <v>35</v>
@@ -1271,7 +1275,7 @@
         <v>39</v>
       </c>
       <c r="E34" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F34" t="s">
         <v>35</v>
@@ -1282,10 +1286,10 @@
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B35" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E35" t="s">
         <v>13</v>
@@ -1294,41 +1298,41 @@
         <v>35</v>
       </c>
       <c r="G35" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K35" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E36" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F36" t="s">
         <v>35</v>
       </c>
       <c r="G36" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="H36" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I36" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B37" t="s">
+        <v>56</v>
+      </c>
+      <c r="C37" t="s">
         <v>57</v>
-      </c>
-      <c r="C37" t="s">
-        <v>58</v>
       </c>
       <c r="E37" t="s">
         <v>11</v>
@@ -1337,18 +1341,18 @@
         <v>9</v>
       </c>
       <c r="G37" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B38" t="s">
+        <v>56</v>
+      </c>
+      <c r="C38" t="s">
         <v>57</v>
-      </c>
-      <c r="C38" t="s">
-        <v>58</v>
       </c>
       <c r="E38" t="s">
         <v>14</v>
@@ -1362,13 +1366,13 @@
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B39" t="s">
+        <v>56</v>
+      </c>
+      <c r="C39" t="s">
         <v>57</v>
-      </c>
-      <c r="C39" t="s">
-        <v>58</v>
       </c>
       <c r="E39" t="s">
         <v>3</v>
@@ -1382,10 +1386,10 @@
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B40" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E40" t="s">
         <v>11</v>
@@ -1394,15 +1398,15 @@
         <v>35</v>
       </c>
       <c r="G40" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B41" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E41" t="s">
         <v>14</v>
@@ -1411,15 +1415,15 @@
         <v>35</v>
       </c>
       <c r="G41" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B42" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E42" t="s">
         <v>3</v>
@@ -1428,27 +1432,27 @@
         <v>35</v>
       </c>
       <c r="G42" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
+        <v>72</v>
+      </c>
+      <c r="B43" t="s">
         <v>73</v>
       </c>
-      <c r="B43" t="s">
+      <c r="C43" t="s">
+        <v>75</v>
+      </c>
+      <c r="D43" t="s">
         <v>74</v>
-      </c>
-      <c r="C43" t="s">
-        <v>76</v>
-      </c>
-      <c r="D43" t="s">
-        <v>75</v>
       </c>
       <c r="E43" t="s">
         <v>13</v>
       </c>
       <c r="F43" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H43" t="s">
         <v>5</v>
@@ -1459,19 +1463,19 @@
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
+        <v>77</v>
+      </c>
+      <c r="B44" t="s">
+        <v>73</v>
+      </c>
+      <c r="D44" t="s">
         <v>78</v>
-      </c>
-      <c r="B44" t="s">
-        <v>74</v>
-      </c>
-      <c r="D44" t="s">
-        <v>79</v>
       </c>
       <c r="E44" t="s">
         <v>13</v>
       </c>
       <c r="F44" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H44" t="s">
         <v>5</v>
@@ -1482,16 +1486,16 @@
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
+        <v>80</v>
+      </c>
+      <c r="B45" t="s">
+        <v>82</v>
+      </c>
+      <c r="D45" t="s">
         <v>81</v>
       </c>
-      <c r="B45" t="s">
-        <v>83</v>
-      </c>
-      <c r="D45" t="s">
-        <v>82</v>
-      </c>
       <c r="E45" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F45" t="s">
         <v>35</v>
@@ -1502,16 +1506,16 @@
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
+        <v>83</v>
+      </c>
+      <c r="B46" t="s">
         <v>84</v>
       </c>
-      <c r="B46" t="s">
+      <c r="C46" t="s">
         <v>85</v>
       </c>
-      <c r="C46" t="s">
+      <c r="D46" t="s">
         <v>86</v>
-      </c>
-      <c r="D46" t="s">
-        <v>87</v>
       </c>
       <c r="E46" t="s">
         <v>13</v>
@@ -1525,13 +1529,13 @@
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
+        <v>87</v>
+      </c>
+      <c r="B47" t="s">
+        <v>89</v>
+      </c>
+      <c r="C47" t="s">
         <v>88</v>
-      </c>
-      <c r="B47" t="s">
-        <v>90</v>
-      </c>
-      <c r="C47" t="s">
-        <v>89</v>
       </c>
       <c r="E47" t="s">
         <v>14</v>
@@ -1545,13 +1549,13 @@
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
+        <v>87</v>
+      </c>
+      <c r="B48" t="s">
+        <v>89</v>
+      </c>
+      <c r="C48" t="s">
         <v>88</v>
-      </c>
-      <c r="B48" t="s">
-        <v>90</v>
-      </c>
-      <c r="C48" t="s">
-        <v>89</v>
       </c>
       <c r="E48" t="s">
         <v>14</v>
@@ -1565,13 +1569,13 @@
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
+        <v>87</v>
+      </c>
+      <c r="B49" t="s">
+        <v>89</v>
+      </c>
+      <c r="C49" t="s">
         <v>88</v>
-      </c>
-      <c r="B49" t="s">
-        <v>90</v>
-      </c>
-      <c r="C49" t="s">
-        <v>89</v>
       </c>
       <c r="E49" t="s">
         <v>30</v>
@@ -1582,22 +1586,22 @@
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
+        <v>90</v>
+      </c>
+      <c r="B50" t="s">
         <v>91</v>
       </c>
-      <c r="B50" t="s">
+      <c r="C50" t="s">
         <v>92</v>
       </c>
-      <c r="C50" t="s">
+      <c r="D50" t="s">
         <v>93</v>
-      </c>
-      <c r="D50" t="s">
-        <v>94</v>
       </c>
       <c r="E50" t="s">
         <v>14</v>
       </c>
       <c r="F50" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="H50" t="s">
         <v>6</v>
@@ -1608,7 +1612,7 @@
         <v>12</v>
       </c>
       <c r="F51" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="H51" t="s">
         <v>6</v>
@@ -1619,14 +1623,14 @@
         <v>3</v>
       </c>
       <c r="F52" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="H52" t="s">
         <v>5</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J42"/>
+  <autoFilter ref="A1:J52"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>